<commit_message>
Cycle functions up to 2B.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C72A2F-E25D-4913-A95C-A36B2BAEE181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97C3209F-083E-4BEC-8D8C-4D9CB1DE1CE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
+    <workbookView xWindow="11340" yWindow="825" windowWidth="16575" windowHeight="14745" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$2360</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$2537</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="191">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -3293,6 +3293,525 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> based off Operand.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>PLP (28)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Read </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> | $0100</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 1. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>P</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> = Operand.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flags, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.H to 0.</t>
+    </r>
+  </si>
+  <si>
+    <t>AND (29)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &amp;= Operand. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 1.</t>
+    </r>
+  </si>
+  <si>
+    <t>ROL (2A)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80). Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &lt;&lt; 1) | </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
     </r>
   </si>
 </sst>
@@ -3888,11 +4407,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C2320"/>
+  <dimension ref="A1:C2487"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
-    <col min="3" max="3" width="88.28515625" customWidth="1"/>
+    <col min="3" max="3" width="93.28515625" customWidth="1"/>
     <col min="4" max="4" width="4.7109375" customWidth="1"/>
     <col min="6" max="8" width="9.140625" customWidth="1"/>
   </cols>
@@ -5359,7 +5878,9 @@
         <v>3.1</v>
       </c>
       <c r="B481" s="9"/>
-      <c r="C481" s="10"/>
+      <c r="C481" s="10" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="482" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A482" s="8">
@@ -7200,21 +7721,21 @@
       <c r="C1249" s="26"/>
     </row>
     <row r="1250" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1250" s="8">
+      <c r="A1250" s="15">
         <v>3.2</v>
       </c>
-      <c r="B1250" s="9"/>
-      <c r="C1250" s="10"/>
+      <c r="B1250" s="16"/>
+      <c r="C1250" s="23"/>
     </row>
     <row r="1251" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1251" s="8">
+      <c r="A1251" s="15">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B1251" s="9"/>
-      <c r="C1251" s="14"/>
+      <c r="B1251" s="16"/>
+      <c r="C1251" s="17"/>
     </row>
     <row r="1252" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1252" s="8">
+      <c r="A1252" s="18">
         <v>4.2</v>
       </c>
       <c r="B1252" s="9" t="s">
@@ -9801,7 +10322,7 @@
       <c r="C2256" s="26"/>
     </row>
     <row r="2257" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2257" s="8">
+      <c r="A2257" s="18">
         <v>5.2</v>
       </c>
       <c r="B2257" s="9" t="s">
@@ -10012,6 +10533,297 @@
       </c>
       <c r="B2320" s="20"/>
       <c r="C2320" s="22"/>
+    </row>
+    <row r="2361" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2361" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2361" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2361" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2362" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2362" s="4"/>
+      <c r="B2362" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2362" s="25"/>
+    </row>
+    <row r="2363" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2363" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2363" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2363" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2364" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2364" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2364" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2364" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2365" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2365" s="9"/>
+      <c r="C2365" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2366" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2366" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B2366" s="9"/>
+      <c r="C2366" s="10"/>
+    </row>
+    <row r="2367" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2367" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B2367" s="9"/>
+      <c r="C2367" s="10"/>
+    </row>
+    <row r="2368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2368" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2368" s="9"/>
+      <c r="C2368" s="10"/>
+    </row>
+    <row r="2369" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2369" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B2369" s="9"/>
+      <c r="C2369" s="10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2370" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2370" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B2370" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="C2370" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2371" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B2371" s="9"/>
+      <c r="C2371" s="14" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="2372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2372" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B2372" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2372" s="14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2373" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2373" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2373" s="20"/>
+      <c r="C2373" s="22"/>
+    </row>
+    <row r="2420" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2420" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B2420" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2420" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2421" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2421" s="4"/>
+      <c r="B2421" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2421" s="6"/>
+    </row>
+    <row r="2422" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2422" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2422" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2422" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2423" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2423" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2423" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2423" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2424" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2424" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2424" s="9"/>
+      <c r="C2424" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2425" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2425" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B2425" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2425" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2426" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2426" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B2426" s="9"/>
+      <c r="C2426" s="10" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2427" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2427" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2427" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2427" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2428" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2428" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2428" s="20"/>
+      <c r="C2428" s="22"/>
+    </row>
+    <row r="2479" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2479" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B2479" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2479" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2480" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2480" s="4"/>
+      <c r="B2480" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2480" s="6"/>
+    </row>
+    <row r="2481" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2481" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2481" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2481" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2482" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2482" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2482" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2482" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2483" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2483" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B2483" s="9"/>
+      <c r="C2483" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2484" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2484" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B2484" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2484" s="10" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2485" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2485" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B2485" s="9"/>
+      <c r="C2485" s="10" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2486" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2486" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B2486" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2486" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2487" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2487" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2487" s="20"/>
+      <c r="C2487" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="33">

</xml_diff>

<commit_message>
Added instructions up to 61.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21507DF-AEA7-4007-8BFF-B95F7253643D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{147C02FF-BB19-4DF8-BCAF-35B663EDEF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -17134,7 +17134,7 @@
       </c>
     </row>
     <row r="4081" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4081" s="8">
+      <c r="A4081" s="18">
         <v>3.2</v>
       </c>
       <c r="B4081" s="9" t="s">
@@ -18931,10 +18931,10 @@
     </row>
     <row r="4899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4899" s="4"/>
-      <c r="B4899" s="24" t="s">
+      <c r="B4899" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="C4899" s="25"/>
+      <c r="C4899" s="32"/>
     </row>
     <row r="4900" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4900" s="12" t="s">
@@ -20773,7 +20773,7 @@
       </c>
     </row>
     <row r="5560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5560" s="8">
+      <c r="A5560" s="18">
         <v>4.2</v>
       </c>
       <c r="B5560" s="9" t="s">
@@ -20811,7 +20811,7 @@
       <c r="C5563" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="78">
+  <mergeCells count="79">
     <mergeCell ref="B5548:C5548"/>
     <mergeCell ref="B5371:C5371"/>
     <mergeCell ref="B5430:C5430"/>
@@ -20826,6 +20826,7 @@
     <mergeCell ref="C5024:C5025"/>
     <mergeCell ref="B4781:C4781"/>
     <mergeCell ref="C4969:C4970"/>
+    <mergeCell ref="B4899:C4899"/>
     <mergeCell ref="C4615:C4616"/>
     <mergeCell ref="B4604:C4604"/>
     <mergeCell ref="B4663:C4663"/>

</xml_diff>

<commit_message>
Updated Windows library, added instructions up to 64.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{147C02FF-BB19-4DF8-BCAF-35B663EDEF99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC56D92A-640B-4C83-8302-3DE023BDC2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$5605</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$5959</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2251" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2407" uniqueCount="310">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -5915,6 +5915,35 @@
     <t>EOR (59)</t>
   </si>
   <si>
+    <t>PHY (5A)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Push </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L onto stack.</t>
+    </r>
+  </si>
+  <si>
     <t>TCD (5B)</t>
   </si>
   <si>
@@ -6112,6 +6141,616 @@
   </si>
   <si>
     <t>EOR (5F)</t>
+  </si>
+  <si>
+    <t>RTS (60)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 1. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to (Operand + 1).</t>
+    </r>
+  </si>
+  <si>
+    <t>ADC (61)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  if (Lo &gt; 9) Lo += 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  CarryToHi = Lo &gt; $0F ? 1 : 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  if (HiSum &gt; 9) HiSum += 6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Result = ui8(((HiSum &amp; 0x0F) &lt;&lt; 4) | (Lo &amp; $0F)).</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag == 0:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = Result &gt; $FF.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag == 1:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  Result = ui16(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L) + ui16(Operand) + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (~(ui16(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L) ^ ui16(Operand)) &amp; (ui16(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L) ^ ui8(Result)) &amp; $80) != 0.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  Result = ui8(Result). </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = Result == $00. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Result &amp; $80) != 0.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  Lo = ui16(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; 0x0F) + ui16(Operand &amp; 0x0F) + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  HiSum = ui16(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L &gt;&gt; 4) + ui16(Operand &gt;&gt; 4) + CarryToHi.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>V</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (~((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L &gt;&gt; 4) ^ (Operand &gt;&gt; 4)) &amp; ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L &gt;&gt; 4) ^ HiSum) &amp; $08) != 0.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = HiSum &gt; $0F.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = Result == $00. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> flag = (Result &amp; $80) != 0.</t>
+    </r>
+  </si>
+  <si>
+    <t>PER (62)</t>
+  </si>
+  <si>
+    <t>Push Operand.H onto stack.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Set Operand to Operand + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dec. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 2.</t>
+    </r>
+  </si>
+  <si>
+    <t>ADC (63)</t>
+  </si>
+  <si>
+    <t>STZ (64)</t>
+  </si>
+  <si>
+    <t>Direct (Write)</t>
+  </si>
+  <si>
+    <t>Write 0.</t>
   </si>
 </sst>
 </file>
@@ -6712,7 +7351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C5563"/>
+  <dimension ref="A1:C5913"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -8172,7 +8811,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B480" s="9" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="C480" s="10" t="s">
         <v>49</v>
@@ -20082,7 +20721,7 @@
         <v>273</v>
       </c>
       <c r="B5311" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C5311" s="3" t="s">
         <v>13</v>
@@ -20127,60 +20766,74 @@
       </c>
     </row>
     <row r="5316" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5316" s="18">
+      <c r="A5316" s="8">
         <v>1.2</v>
       </c>
-      <c r="B5316" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5316" s="10" t="s">
-        <v>73</v>
-      </c>
+      <c r="B5316" s="9"/>
+      <c r="C5316" s="10"/>
     </row>
     <row r="5317" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5317" s="8">
         <v>2.1</v>
       </c>
       <c r="B5317" s="9"/>
-      <c r="C5317" s="10" t="s">
+      <c r="C5317" s="10"/>
+    </row>
+    <row r="5318" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5318" s="18">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5318" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C5318" s="10" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="5318" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5318" s="8">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="B5318" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5318" s="10" t="s">
+    <row r="5319" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5319" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5319" s="9"/>
+      <c r="C5319" s="10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5320" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5320" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B5320" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5320" s="10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5319" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5319" s="19" t="s">
+    <row r="5321" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5321" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B5319" s="20"/>
-      <c r="C5319" s="22"/>
+      <c r="B5321" s="20"/>
+      <c r="C5321" s="22"/>
     </row>
     <row r="5370" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5370" s="1" t="s">
         <v>275</v>
       </c>
       <c r="B5370" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C5370" s="3" t="s">
-        <v>82</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5371" s="4"/>
-      <c r="B5371" s="31" t="s">
-        <v>139</v>
-      </c>
-      <c r="C5371" s="32"/>
+      <c r="B5371" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5371" s="25"/>
     </row>
     <row r="5372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5372" s="12" t="s">
@@ -20214,14 +20867,14 @@
       </c>
     </row>
     <row r="5375" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5375" s="8">
+      <c r="A5375" s="18">
         <v>1.2</v>
       </c>
       <c r="B5375" s="9" t="s">
         <v>72</v>
       </c>
       <c r="C5375" s="10" t="s">
-        <v>16</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5376" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20230,7 +20883,7 @@
       </c>
       <c r="B5376" s="9"/>
       <c r="C5376" s="10" t="s">
-        <v>56</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5377" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20241,71 +20894,31 @@
         <v>72</v>
       </c>
       <c r="C5377" s="10" t="s">
-        <v>276</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5378" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5378" s="8">
-        <v>3.1</v>
-      </c>
-      <c r="B5378" s="9"/>
-      <c r="C5378" s="10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5379" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5379" s="18">
-        <v>3.2</v>
-      </c>
-      <c r="B5379" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5379" s="10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5380" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5380" s="8">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="B5380" s="9"/>
-      <c r="C5380" s="10" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="5381" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5381" s="8">
-        <v>4.2</v>
-      </c>
-      <c r="B5381" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5381" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5382" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5382" s="19" t="s">
+      <c r="A5378" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B5382" s="20"/>
-      <c r="C5382" s="22"/>
+      <c r="B5378" s="20"/>
+      <c r="C5378" s="22"/>
     </row>
     <row r="5429" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5429" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5429" s="2" t="s">
         <v>24</v>
       </c>
       <c r="C5429" s="3" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5430" s="4"/>
       <c r="B5430" s="31" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="C5430" s="32"/>
     </row>
@@ -20345,10 +20958,10 @@
         <v>1.2</v>
       </c>
       <c r="B5434" s="9" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="C5434" s="10" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5435" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20365,10 +20978,10 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B5436" s="9" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="C5436" s="10" t="s">
-        <v>37</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5437" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20377,88 +20990,53 @@
       </c>
       <c r="B5437" s="9"/>
       <c r="C5437" s="10" t="s">
-        <v>116</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5438" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5438" s="8"/>
-      <c r="B5438" s="9"/>
+      <c r="A5438" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B5438" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="C5438" s="10" t="s">
-        <v>125</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5439" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5439" s="8"/>
+      <c r="A5439" s="8">
+        <v>4.0999999999999996</v>
+      </c>
       <c r="B5439" s="9"/>
       <c r="C5439" s="10" t="s">
         <v>279</v>
       </c>
     </row>
     <row r="5440" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5440" s="8"/>
-      <c r="B5440" s="9"/>
+      <c r="A5440" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5440" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="C5440" s="10" t="s">
-        <v>91</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5441" s="15">
-        <v>3.2</v>
-      </c>
-      <c r="B5441" s="16"/>
-      <c r="C5441" s="23"/>
-    </row>
-    <row r="5442" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5442" s="15">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="B5442" s="16"/>
-      <c r="C5442" s="23"/>
-    </row>
-    <row r="5443" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5443" s="18">
-        <v>4.2</v>
-      </c>
-      <c r="B5443" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5443" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5444" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5444" s="8">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B5444" s="9"/>
-      <c r="C5444" s="10" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="5445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5445" s="8">
-        <v>5.2</v>
-      </c>
-      <c r="B5445" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5445" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5446" s="19" t="s">
+      <c r="A5441" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B5446" s="20"/>
-      <c r="C5446" s="22"/>
+      <c r="B5441" s="20"/>
+      <c r="C5441" s="22"/>
     </row>
     <row r="5488" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5488" s="1" t="s">
         <v>280</v>
       </c>
       <c r="B5488" s="2" t="s">
-        <v>98</v>
+        <v>24</v>
       </c>
       <c r="C5488" s="3" t="s">
         <v>32</v>
@@ -20467,7 +21045,7 @@
     <row r="5489" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5489" s="4"/>
       <c r="B5489" s="31" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C5489" s="32"/>
     </row>
@@ -20507,7 +21085,7 @@
         <v>1.2</v>
       </c>
       <c r="B5493" s="9" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="C5493" s="10" t="s">
         <v>31</v>
@@ -20527,7 +21105,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B5495" s="9" t="s">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="C5495" s="10" t="s">
         <v>37</v>
@@ -20539,131 +21117,97 @@
       </c>
       <c r="B5496" s="9"/>
       <c r="C5496" s="10" t="s">
-        <v>168</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5497" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5497" s="8"/>
       <c r="B5497" s="9"/>
       <c r="C5497" s="10" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
     </row>
     <row r="5498" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5498" s="8"/>
       <c r="B5498" s="9"/>
       <c r="C5498" s="10" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="5499" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5499" s="8"/>
+      <c r="B5499" s="9"/>
+      <c r="C5499" s="10" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="5499" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5499" s="8">
+    <row r="5500" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5500" s="15">
         <v>3.2</v>
       </c>
-      <c r="B5499" s="9"/>
-      <c r="C5499" s="10"/>
-    </row>
-    <row r="5500" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5500" s="8">
+      <c r="B5500" s="16"/>
+      <c r="C5500" s="23"/>
+    </row>
+    <row r="5501" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5501" s="15">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B5500" s="9"/>
-      <c r="C5500" s="10"/>
-    </row>
-    <row r="5501" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5501" s="8">
+      <c r="B5501" s="16"/>
+      <c r="C5501" s="23"/>
+    </row>
+    <row r="5502" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5502" s="18">
         <v>4.2</v>
       </c>
-      <c r="B5501" s="9" t="s">
+      <c r="B5502" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C5501" s="10" t="s">
+      <c r="C5502" s="10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5502" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5502" s="8">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="B5502" s="9"/>
-      <c r="C5502" s="10"/>
     </row>
     <row r="5503" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5503" s="8">
-        <v>5.2</v>
-      </c>
-      <c r="B5503" s="9" t="s">
-        <v>128</v>
-      </c>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B5503" s="9"/>
       <c r="C5503" s="10" t="s">
-        <v>47</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5504" s="8">
-        <v>6.1</v>
-      </c>
-      <c r="B5504" s="9"/>
-      <c r="C5504" s="30" t="s">
-        <v>232</v>
+        <v>5.2</v>
+      </c>
+      <c r="B5504" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5504" s="10" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5505" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5505" s="8"/>
-      <c r="B5505" s="9"/>
-      <c r="C5505" s="30"/>
-    </row>
-    <row r="5506" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5506" s="18">
-        <v>6.2</v>
-      </c>
-      <c r="B5506" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5506" s="10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5507" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5507" s="8">
-        <v>7.1</v>
-      </c>
-      <c r="B5507" s="9"/>
-      <c r="C5507" s="10"/>
-    </row>
-    <row r="5508" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5508" s="8">
-        <v>7.2</v>
-      </c>
-      <c r="B5508" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5508" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5509" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5509" s="19" t="s">
+      <c r="A5505" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B5509" s="20"/>
-      <c r="C5509" s="22"/>
+      <c r="B5505" s="20"/>
+      <c r="C5505" s="22"/>
     </row>
     <row r="5547" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5547" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B5547" s="2" t="s">
-        <v>19</v>
+        <v>98</v>
       </c>
       <c r="C5547" s="3" t="s">
-        <v>82</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5548" s="4"/>
       <c r="B5548" s="31" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C5548" s="32"/>
     </row>
@@ -20735,45 +21279,39 @@
       </c>
       <c r="B5555" s="9"/>
       <c r="C5555" s="10" t="s">
-        <v>56</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5556" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5556" s="8">
-        <v>3.2</v>
-      </c>
-      <c r="B5556" s="9" t="s">
-        <v>72</v>
-      </c>
+      <c r="A5556" s="8"/>
+      <c r="B5556" s="9"/>
       <c r="C5556" s="10" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5557" s="8">
-        <v>4.0999999999999996</v>
-      </c>
+      <c r="A5557" s="8"/>
       <c r="B5557" s="9"/>
       <c r="C5557" s="10" t="s">
-        <v>168</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5558" s="8"/>
+      <c r="A5558" s="8">
+        <v>3.2</v>
+      </c>
       <c r="B5558" s="9"/>
-      <c r="C5558" s="10" t="s">
-        <v>102</v>
-      </c>
+      <c r="C5558" s="10"/>
     </row>
     <row r="5559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5559" s="8"/>
+      <c r="A5559" s="8">
+        <v>4.0999999999999996</v>
+      </c>
       <c r="B5559" s="9"/>
-      <c r="C5559" s="10" t="s">
-        <v>118</v>
-      </c>
+      <c r="C5559" s="10"/>
     </row>
     <row r="5560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5560" s="18">
+      <c r="A5560" s="8">
         <v>4.2</v>
       </c>
       <c r="B5560" s="9" t="s">
@@ -20788,35 +21326,1164 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B5561" s="9"/>
-      <c r="C5561" s="10" t="s">
-        <v>222</v>
-      </c>
+      <c r="C5561" s="10"/>
     </row>
     <row r="5562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5562" s="8">
         <v>5.2</v>
       </c>
       <c r="B5562" s="9" t="s">
-        <v>72</v>
+        <v>128</v>
       </c>
       <c r="C5562" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5563" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B5563" s="9"/>
+      <c r="C5563" s="30" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5564" s="8"/>
+      <c r="B5564" s="9"/>
+      <c r="C5564" s="30"/>
+    </row>
+    <row r="5565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5565" s="18">
+        <v>6.2</v>
+      </c>
+      <c r="B5565" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5565" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5566" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="B5566" s="9"/>
+      <c r="C5566" s="10"/>
+    </row>
+    <row r="5567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5567" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="B5567" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5567" s="10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5563" s="19" t="s">
+    <row r="5568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5568" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B5563" s="20"/>
-      <c r="C5563" s="22"/>
+      <c r="B5568" s="20"/>
+      <c r="C5568" s="22"/>
+    </row>
+    <row r="5606" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5606" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="B5606" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5606" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5607" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5607" s="4"/>
+      <c r="B5607" s="31" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5607" s="32"/>
+    </row>
+    <row r="5608" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5608" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5608" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5608" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5609" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5609" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5609" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5609" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5610" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5610" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5610" s="9"/>
+      <c r="C5610" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5611" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5611" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5611" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5611" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5612" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5612" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B5612" s="9"/>
+      <c r="C5612" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5613" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5613" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5613" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5613" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5614" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5614" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5614" s="9"/>
+      <c r="C5614" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5615" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5615" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B5615" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5615" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5616" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5616" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5616" s="9"/>
+      <c r="C5616" s="10" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="5617" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5617" s="8"/>
+      <c r="B5617" s="9"/>
+      <c r="C5617" s="10" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="5618" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5618" s="8"/>
+      <c r="B5618" s="9"/>
+      <c r="C5618" s="10" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="5619" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5619" s="18">
+        <v>4.2</v>
+      </c>
+      <c r="B5619" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5619" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5620" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5620" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B5620" s="9"/>
+      <c r="C5620" s="10" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5621" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5621" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B5621" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5621" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5622" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5622" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5622" s="20"/>
+      <c r="C5622" s="22"/>
+    </row>
+    <row r="5665" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5665" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="B5665" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5665" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5666" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5666" s="4"/>
+      <c r="B5666" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5666" s="25"/>
+    </row>
+    <row r="5667" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5667" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5667" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5667" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5668" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5668" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5668" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5668" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5669" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5669" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5669" s="9"/>
+      <c r="C5669" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5670" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5670" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5670" s="9"/>
+      <c r="C5670" s="10"/>
+    </row>
+    <row r="5671" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5671" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B5671" s="9"/>
+      <c r="C5671" s="10"/>
+    </row>
+    <row r="5672" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5672" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5672" s="9"/>
+      <c r="C5672" s="10"/>
+    </row>
+    <row r="5673" spans="1:3" s="28" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5673" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5673" s="9"/>
+      <c r="C5673" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="5674" spans="1:3" s="28" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5674" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B5674" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="C5674" s="10" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="5675" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5675" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5675" s="9"/>
+      <c r="C5675" s="10"/>
+    </row>
+    <row r="5676" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5676" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5676" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="C5676" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5677" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5677" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B5677" s="9"/>
+      <c r="C5677" s="10"/>
+    </row>
+    <row r="5678" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5678" s="18">
+        <v>5.2</v>
+      </c>
+      <c r="B5678" s="9"/>
+      <c r="C5678" s="10"/>
+    </row>
+    <row r="5679" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5679" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B5679" s="9"/>
+      <c r="C5679" s="10" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="5680" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5680" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B5680" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5680" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5681" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5681" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5681" s="20"/>
+      <c r="C5681" s="22"/>
+    </row>
+    <row r="5724" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5724" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B5724" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5724" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5725" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5725" s="4"/>
+      <c r="B5725" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5725" s="32"/>
+    </row>
+    <row r="5726" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5726" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5726" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5726" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5727" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5727" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5727" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5727" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5728" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5728" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5728" s="9"/>
+      <c r="C5728" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5729" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5729" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5729" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5729" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5730" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5730" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B5730" s="9"/>
+      <c r="C5730" s="10" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5731" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5731" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5731" s="9"/>
+      <c r="C5731" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5732" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5732" s="15">
+        <v>3.1</v>
+      </c>
+      <c r="B5732" s="16"/>
+      <c r="C5732" s="23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5733" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5733" s="15">
+        <v>3.2</v>
+      </c>
+      <c r="B5733" s="16"/>
+      <c r="C5733" s="23"/>
+    </row>
+    <row r="5734" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5734" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5734" s="9"/>
+      <c r="C5734" s="10"/>
+    </row>
+    <row r="5735" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5735" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5735" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5735" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5736" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5736" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B5736" s="9"/>
+      <c r="C5736" s="10"/>
+    </row>
+    <row r="5737" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5737" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B5737" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5737" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5738" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5738" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B5738" s="9"/>
+      <c r="C5738" s="10"/>
+    </row>
+    <row r="5739" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5739" s="18">
+        <v>6.2</v>
+      </c>
+      <c r="B5739" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5739" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5740" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5740" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="B5740" s="9"/>
+      <c r="C5740" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="5741" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5741" s="8"/>
+      <c r="B5741" s="9"/>
+      <c r="C5741" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5742" s="8"/>
+      <c r="B5742" s="9"/>
+      <c r="C5742" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5743" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5743" s="8"/>
+      <c r="B5743" s="9"/>
+      <c r="C5743" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="5744" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5744" s="8"/>
+      <c r="B5744" s="9"/>
+      <c r="C5744" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="5745" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5745" s="8"/>
+      <c r="B5745" s="9"/>
+      <c r="C5745" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5746" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5746" s="8"/>
+      <c r="B5746" s="9"/>
+      <c r="C5746" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5747" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5747" s="8"/>
+      <c r="B5747" s="9"/>
+      <c r="C5747" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5748" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5748" s="8"/>
+      <c r="B5748" s="9"/>
+      <c r="C5748" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="5749" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5749" s="8"/>
+      <c r="B5749" s="9"/>
+      <c r="C5749" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="5750" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5750" s="8"/>
+      <c r="B5750" s="9"/>
+      <c r="C5750" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="5751" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5751" s="8"/>
+      <c r="B5751" s="9"/>
+      <c r="C5751" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5752" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5752" s="8"/>
+      <c r="B5752" s="9"/>
+      <c r="C5752" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5753" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5753" s="8"/>
+      <c r="B5753" s="9"/>
+      <c r="C5753" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5754" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5754" s="8"/>
+      <c r="B5754" s="9"/>
+      <c r="C5754" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="5755" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5755" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="B5755" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5755" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5756" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5756" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5756" s="20"/>
+      <c r="C5756" s="22"/>
+    </row>
+    <row r="5783" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5783" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B5783" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5783" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5784" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5784" s="4"/>
+      <c r="B5784" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5784" s="25"/>
+    </row>
+    <row r="5785" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5785" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5785" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5785" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5786" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5786" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5786" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5786" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5787" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5787" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5787" s="9"/>
+      <c r="C5787" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5788" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5788" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5788" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5788" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5789" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5789" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B5789" s="9"/>
+      <c r="C5789" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5790" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5790" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5790" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5790" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5791" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5791" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5791" s="9"/>
+      <c r="C5791" s="10" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="5792" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5792" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B5792" s="9"/>
+      <c r="C5792" s="10"/>
+    </row>
+    <row r="5793" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5793" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5793" s="9"/>
+      <c r="C5793" s="10"/>
+    </row>
+    <row r="5794" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5794" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5794" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C5794" s="10" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="5795" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5795" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B5795" s="9"/>
+      <c r="C5795" s="10"/>
+    </row>
+    <row r="5796" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5796" s="18">
+        <v>5.2</v>
+      </c>
+      <c r="B5796" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="C5796" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5797" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5797" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B5797" s="9"/>
+      <c r="C5797" s="10" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="5798" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5798" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B5798" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5798" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5799" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5799" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5799" s="20"/>
+      <c r="C5799" s="22"/>
+    </row>
+    <row r="5842" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5842" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="B5842" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5842" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5843" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5843" s="4"/>
+      <c r="B5843" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5843" s="25"/>
+    </row>
+    <row r="5844" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5844" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5844" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5844" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5845" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5845" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5845" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5845" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5846" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5846" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5846" s="9"/>
+      <c r="C5846" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5847" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5847" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5847" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5847" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5848" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5848" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B5848" s="9"/>
+      <c r="C5848" s="10" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5849" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5849" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5849" s="9"/>
+      <c r="C5849" s="10"/>
+    </row>
+    <row r="5850" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5850" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5850" s="9"/>
+      <c r="C5850" s="10"/>
+    </row>
+    <row r="5851" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5851" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B5851" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5851" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5852" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5852" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5852" s="9"/>
+      <c r="C5852" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="5853" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5853" s="8"/>
+      <c r="B5853" s="9"/>
+      <c r="C5853" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5854" s="8"/>
+      <c r="B5854" s="9"/>
+      <c r="C5854" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5855" s="8"/>
+      <c r="B5855" s="9"/>
+      <c r="C5855" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="5856" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5856" s="8"/>
+      <c r="B5856" s="9"/>
+      <c r="C5856" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="5857" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5857" s="8"/>
+      <c r="B5857" s="9"/>
+      <c r="C5857" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5858" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5858" s="8"/>
+      <c r="B5858" s="9"/>
+      <c r="C5858" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5859" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5859" s="8"/>
+      <c r="B5859" s="9"/>
+      <c r="C5859" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5860" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5860" s="8"/>
+      <c r="B5860" s="9"/>
+      <c r="C5860" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="5861" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5861" s="8"/>
+      <c r="B5861" s="9"/>
+      <c r="C5861" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="5862" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5862" s="8"/>
+      <c r="B5862" s="9"/>
+      <c r="C5862" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="5863" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5863" s="8"/>
+      <c r="B5863" s="9"/>
+      <c r="C5863" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5864" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5864" s="8"/>
+      <c r="B5864" s="9"/>
+      <c r="C5864" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5865" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5865" s="8"/>
+      <c r="B5865" s="9"/>
+      <c r="C5865" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5866" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5866" s="8"/>
+      <c r="B5866" s="9"/>
+      <c r="C5866" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="5867" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5867" s="8"/>
+      <c r="B5867" s="9"/>
+      <c r="C5867" s="10"/>
+    </row>
+    <row r="5868" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5868" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5868" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5868" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5869" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5869" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5869" s="20"/>
+      <c r="C5869" s="22"/>
+    </row>
+    <row r="5901" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5901" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B5901" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5901" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5902" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5902" s="4"/>
+      <c r="B5902" s="24" t="s">
+        <v>308</v>
+      </c>
+      <c r="C5902" s="25"/>
+    </row>
+    <row r="5903" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5903" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5903" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5903" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5904" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5904" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5904" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5904" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5905" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5905" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5905" s="9"/>
+      <c r="C5905" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5906" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5906" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5906" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5906" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5907" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5907" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B5907" s="16"/>
+      <c r="C5907" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5908" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5908" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5908" s="16"/>
+      <c r="C5908" s="23"/>
+    </row>
+    <row r="5909" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5909" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5909" s="9"/>
+      <c r="C5909" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5910" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5910" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B5910" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5910" s="10" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="5911" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5911" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5911" s="9"/>
+      <c r="C5911" s="10"/>
+    </row>
+    <row r="5912" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5912" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5912" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5912" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5913" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5913" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5913" s="20"/>
+      <c r="C5913" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="79">
-    <mergeCell ref="B5548:C5548"/>
-    <mergeCell ref="B5371:C5371"/>
+  <mergeCells count="80">
+    <mergeCell ref="B5725:C5725"/>
+    <mergeCell ref="B5607:C5607"/>
     <mergeCell ref="B5430:C5430"/>
     <mergeCell ref="B5489:C5489"/>
-    <mergeCell ref="C5504:C5505"/>
+    <mergeCell ref="B5548:C5548"/>
+    <mergeCell ref="C5563:C5564"/>
     <mergeCell ref="B5135:C5135"/>
     <mergeCell ref="B5145:B5147"/>
     <mergeCell ref="B5149:B5151"/>

</xml_diff>

<commit_message>
Added instructions up to 6F.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC56D92A-640B-4C83-8302-3DE023BDC2F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94886885-B220-4532-9DAD-FCA78D6CA6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$5959</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$6608</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2407" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2724" uniqueCount="332">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -6751,6 +6751,718 @@
   </si>
   <si>
     <t>Write 0.</t>
+  </si>
+  <si>
+    <t>ADC (65)</t>
+  </si>
+  <si>
+    <t>ROR (66)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $01). Perform Operand.L = (Operand.L &gt;&gt; 1) | (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;&lt; 7). Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (Operand.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off Operand.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>ADC (67)</t>
+  </si>
+  <si>
+    <t>PLA (68)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L to Operand.L. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Operand. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.H &amp; $80). Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>D</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>ADC (69)</t>
+  </si>
+  <si>
+    <t>ROR (6A)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $01). Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L &gt;&gt; 1) | (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;&lt; 7). Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>RTL (6B)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Store as </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 3. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to (Operand + 1). Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Bank.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L | $0100)+3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read u8(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L+2) | $0100</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read u8(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L+1) | $0100</t>
+    </r>
+  </si>
+  <si>
+    <t>JMP (6C)</t>
+  </si>
+  <si>
+    <t>Absolute Indirect</t>
+  </si>
+  <si>
+    <t>Read Pointer</t>
+  </si>
+  <si>
+    <t>Read Pointer + 1</t>
+  </si>
+  <si>
+    <t>ADC (6D)</t>
+  </si>
+  <si>
+    <t>ROR (6E)</t>
+  </si>
+  <si>
+    <t>ADC (6F)</t>
   </si>
 </sst>
 </file>
@@ -7351,7 +8063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C5913"/>
+  <dimension ref="A1:C6578"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -22333,27 +23045,22 @@
       </c>
     </row>
     <row r="5867" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5867" s="8"/>
-      <c r="B5867" s="9"/>
-      <c r="C5867" s="10"/>
+      <c r="A5867" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5867" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5867" s="10" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5868" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5868" s="8">
-        <v>4.2</v>
-      </c>
-      <c r="B5868" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5868" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5869" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5869" s="19" t="s">
+      <c r="A5868" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B5869" s="20"/>
-      <c r="C5869" s="22"/>
+      <c r="B5868" s="20"/>
+      <c r="C5868" s="22"/>
     </row>
     <row r="5901" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5901" s="1" t="s">
@@ -22476,9 +23183,2002 @@
       <c r="B5913" s="20"/>
       <c r="C5913" s="22"/>
     </row>
+    <row r="5960" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5960" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B5960" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5960" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5961" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5961" s="4"/>
+      <c r="B5961" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5961" s="25"/>
+    </row>
+    <row r="5962" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5962" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5962" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5962" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5963" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5963" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5963" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5963" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5964" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B5964" s="9"/>
+      <c r="C5964" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5965" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5965" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B5965" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5965" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5966" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5966" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B5966" s="16"/>
+      <c r="C5966" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5967" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5967" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B5967" s="16"/>
+      <c r="C5967" s="23"/>
+    </row>
+    <row r="5968" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5968" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B5968" s="9"/>
+      <c r="C5968" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5969" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5969" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B5969" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5969" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5970" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5970" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B5970" s="9"/>
+      <c r="C5970" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="5971" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5971" s="8"/>
+      <c r="B5971" s="9"/>
+      <c r="C5971" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5972" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5972" s="8"/>
+      <c r="B5972" s="9"/>
+      <c r="C5972" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5973" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5973" s="8"/>
+      <c r="B5973" s="9"/>
+      <c r="C5973" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="5974" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5974" s="8"/>
+      <c r="B5974" s="9"/>
+      <c r="C5974" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="5975" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5975" s="8"/>
+      <c r="B5975" s="9"/>
+      <c r="C5975" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="5976" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5976" s="8"/>
+      <c r="B5976" s="9"/>
+      <c r="C5976" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5977" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5977" s="8"/>
+      <c r="B5977" s="9"/>
+      <c r="C5977" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="5978" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5978" s="8"/>
+      <c r="B5978" s="9"/>
+      <c r="C5978" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="5979" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5979" s="8"/>
+      <c r="B5979" s="9"/>
+      <c r="C5979" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="5980" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5980" s="8"/>
+      <c r="B5980" s="9"/>
+      <c r="C5980" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="5981" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5981" s="8"/>
+      <c r="B5981" s="9"/>
+      <c r="C5981" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="5982" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5982" s="8"/>
+      <c r="B5982" s="9"/>
+      <c r="C5982" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5983" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5983" s="8"/>
+      <c r="B5983" s="9"/>
+      <c r="C5983" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="5984" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5984" s="8"/>
+      <c r="B5984" s="9"/>
+      <c r="C5984" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="5985" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5985" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B5985" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5985" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5986" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5986" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5986" s="20"/>
+      <c r="C5986" s="22"/>
+    </row>
+    <row r="6019" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6019" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="B6019" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6019" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6020" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6020" s="4"/>
+      <c r="B6020" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6020" s="32"/>
+    </row>
+    <row r="6021" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6021" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6021" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6021" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6022" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6022" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6022" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6022" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6023" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6023" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6023" s="9"/>
+      <c r="C6023" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6024" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6024" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6024" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6024" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6025" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6025" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B6025" s="16"/>
+      <c r="C6025" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6026" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6026" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6026" s="16"/>
+      <c r="C6026" s="23"/>
+    </row>
+    <row r="6027" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6027" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6027" s="9"/>
+      <c r="C6027" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6028" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6028" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B6028" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6028" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6029" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6029" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6029" s="9"/>
+      <c r="C6029" s="10"/>
+    </row>
+    <row r="6030" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6030" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6030" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6030" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6031" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6031" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B6031" s="9"/>
+      <c r="C6031" s="30" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6032" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6032" s="8"/>
+      <c r="B6032" s="9"/>
+      <c r="C6032" s="30"/>
+    </row>
+    <row r="6033" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6033" s="18">
+        <v>5.2</v>
+      </c>
+      <c r="B6033" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6033" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6034" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B6034" s="9"/>
+      <c r="C6034" s="10"/>
+    </row>
+    <row r="6035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6035" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B6035" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6035" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6036" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6036" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6036" s="20"/>
+      <c r="C6036" s="21"/>
+    </row>
+    <row r="6078" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6078" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B6078" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6078" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6079" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6079" s="4"/>
+      <c r="B6079" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6079" s="25"/>
+    </row>
+    <row r="6080" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6080" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6080" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6080" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6081" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6081" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6081" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6081" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6082" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6082" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6082" s="9"/>
+      <c r="C6082" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6083" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6083" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6083" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6083" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6084" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6084" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B6084" s="16"/>
+      <c r="C6084" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6085" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6085" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6085" s="16"/>
+      <c r="C6085" s="23"/>
+    </row>
+    <row r="6086" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6086" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6086" s="9"/>
+      <c r="C6086" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6087" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6087" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B6087" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6087" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6088" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6088" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6088" s="9"/>
+      <c r="C6088" s="10"/>
+    </row>
+    <row r="6089" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6089" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6089" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6089" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6090" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B6090" s="9"/>
+      <c r="C6090" s="10"/>
+    </row>
+    <row r="6091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6091" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B6091" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6091" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6092" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6092" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B6092" s="9"/>
+      <c r="C6092" s="10"/>
+    </row>
+    <row r="6093" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6093" s="18">
+        <v>6.2</v>
+      </c>
+      <c r="B6093" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6093" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6094" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6094" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="B6094" s="9"/>
+      <c r="C6094" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6095" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6095" s="8"/>
+      <c r="B6095" s="9"/>
+      <c r="C6095" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="6096" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6096" s="8"/>
+      <c r="B6096" s="9"/>
+      <c r="C6096" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6097" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6097" s="8"/>
+      <c r="B6097" s="9"/>
+      <c r="C6097" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6098" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6098" s="8"/>
+      <c r="B6098" s="9"/>
+      <c r="C6098" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6099" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6099" s="8"/>
+      <c r="B6099" s="9"/>
+      <c r="C6099" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="6100" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6100" s="8"/>
+      <c r="B6100" s="9"/>
+      <c r="C6100" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6101" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6101" s="8"/>
+      <c r="B6101" s="9"/>
+      <c r="C6101" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="6102" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6102" s="8"/>
+      <c r="B6102" s="9"/>
+      <c r="C6102" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="6103" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6103" s="8"/>
+      <c r="B6103" s="9"/>
+      <c r="C6103" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6104" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6104" s="8"/>
+      <c r="B6104" s="9"/>
+      <c r="C6104" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="6105" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6105" s="8"/>
+      <c r="B6105" s="9"/>
+      <c r="C6105" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="6106" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6106" s="8"/>
+      <c r="B6106" s="9"/>
+      <c r="C6106" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6107" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6107" s="8"/>
+      <c r="B6107" s="9"/>
+      <c r="C6107" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="6108" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6108" s="8"/>
+      <c r="B6108" s="9"/>
+      <c r="C6108" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="6109" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6109" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="B6109" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6109" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6110" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6110" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6110" s="20"/>
+      <c r="C6110" s="22"/>
+    </row>
+    <row r="6137" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6137" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B6137" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6137" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6138" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6138" s="4"/>
+      <c r="B6138" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6138" s="25"/>
+    </row>
+    <row r="6139" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6139" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6139" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6139" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6140" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6140" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6140" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6140" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6141" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6141" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6141" s="9"/>
+      <c r="C6141" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6142" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6142" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6142" s="9"/>
+      <c r="C6142" s="10"/>
+    </row>
+    <row r="6143" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6143" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6143" s="9"/>
+      <c r="C6143" s="10"/>
+    </row>
+    <row r="6144" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6144" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6144" s="9"/>
+      <c r="C6144" s="10"/>
+    </row>
+    <row r="6145" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6145" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6145" s="9"/>
+      <c r="C6145" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6146" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B6146" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="C6146" s="10" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="6147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6147" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6147" s="9"/>
+      <c r="C6147" s="35" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="6148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6148" s="8"/>
+      <c r="B6148" s="9"/>
+      <c r="C6148" s="35"/>
+    </row>
+    <row r="6149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6149" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6149" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6149" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6150" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6150" s="20"/>
+      <c r="C6150" s="22"/>
+    </row>
+    <row r="6196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6196" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B6196" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6196" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6197" s="4"/>
+      <c r="B6197" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6197" s="25"/>
+    </row>
+    <row r="6198" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6198" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6198" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6198" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6199" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6199" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6199" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6199" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6200" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6200" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6200" s="9"/>
+      <c r="C6200" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6201" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6201" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B6201" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6201" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6202" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6202" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6202" s="9"/>
+      <c r="C6202" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6203" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6203" s="8"/>
+      <c r="B6203" s="9"/>
+      <c r="C6203" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="6204" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6204" s="8"/>
+      <c r="B6204" s="9"/>
+      <c r="C6204" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6205" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6205" s="8"/>
+      <c r="B6205" s="9"/>
+      <c r="C6205" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6206" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6206" s="8"/>
+      <c r="B6206" s="9"/>
+      <c r="C6206" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6207" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6207" s="8"/>
+      <c r="B6207" s="9"/>
+      <c r="C6207" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="6208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6208" s="8"/>
+      <c r="B6208" s="9"/>
+      <c r="C6208" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6209" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6209" s="8"/>
+      <c r="B6209" s="9"/>
+      <c r="C6209" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="6210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6210" s="8"/>
+      <c r="B6210" s="9"/>
+      <c r="C6210" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="6211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6211" s="8"/>
+      <c r="B6211" s="9"/>
+      <c r="C6211" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6212" s="8"/>
+      <c r="B6212" s="9"/>
+      <c r="C6212" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="6213" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6213" s="8"/>
+      <c r="B6213" s="9"/>
+      <c r="C6213" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="6214" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6214" s="8"/>
+      <c r="B6214" s="9"/>
+      <c r="C6214" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6215" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6215" s="8"/>
+      <c r="B6215" s="9"/>
+      <c r="C6215" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="6216" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6216" s="8"/>
+      <c r="B6216" s="9"/>
+      <c r="C6216" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="6217" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6217" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6217" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6217" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6218" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6218" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6218" s="20"/>
+      <c r="C6218" s="22"/>
+    </row>
+    <row r="6255" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6255" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="B6255" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6255" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6256" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6256" s="4"/>
+      <c r="B6256" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6256" s="25"/>
+    </row>
+    <row r="6257" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6257" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6257" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6257" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6258" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6258" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6258" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6258" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6259" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6259" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6259" s="9"/>
+      <c r="C6259" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6260" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6260" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B6260" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6260" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6261" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6261" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6261" s="9"/>
+      <c r="C6261" s="10" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="6262" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6262" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6262" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6262" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6263" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6263" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6263" s="20"/>
+      <c r="C6263" s="22"/>
+    </row>
+    <row r="6314" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6314" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="B6314" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6314" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6315" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6315" s="4"/>
+      <c r="B6315" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6315" s="25"/>
+    </row>
+    <row r="6316" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6316" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6316" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6316" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6317" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6317" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6317" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6317" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6318" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6318" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6318" s="9"/>
+      <c r="C6318" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6319" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6319" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6319" s="9"/>
+      <c r="C6319" s="10"/>
+    </row>
+    <row r="6320" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6320" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6320" s="9"/>
+      <c r="C6320" s="10"/>
+    </row>
+    <row r="6321" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6321" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6321" s="9"/>
+      <c r="C6321" s="10"/>
+    </row>
+    <row r="6322" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6322" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6322" s="9"/>
+      <c r="C6322" s="10"/>
+    </row>
+    <row r="6323" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6323" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B6323" s="9" t="s">
+        <v>324</v>
+      </c>
+      <c r="C6323" s="10" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="6324" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6324" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6324" s="9"/>
+      <c r="C6324" s="10"/>
+    </row>
+    <row r="6325" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6325" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6325" s="9" t="s">
+        <v>323</v>
+      </c>
+      <c r="C6325" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6326" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6326" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B6326" s="9"/>
+      <c r="C6326" s="10"/>
+    </row>
+    <row r="6327" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6327" s="18">
+        <v>5.2</v>
+      </c>
+      <c r="B6327" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="C6327" s="10" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="6328" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6328" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B6328" s="9"/>
+      <c r="C6328" s="10" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="6329" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6329" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B6329" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6329" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6330" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6330" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6330" s="20"/>
+      <c r="C6330" s="22"/>
+    </row>
+    <row r="6373" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6373" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="B6373" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6373" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6374" s="4"/>
+      <c r="B6374" s="24" t="s">
+        <v>326</v>
+      </c>
+      <c r="C6374" s="25"/>
+    </row>
+    <row r="6375" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6375" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6375" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6375" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6376" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6376" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6376" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6376" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6377" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6377" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6377" s="9"/>
+      <c r="C6377" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6378" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6378" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6378" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6378" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6379" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6379" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6379" s="9"/>
+      <c r="C6379" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6380" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6380" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6380" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6380" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6381" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6381" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6381" s="9"/>
+      <c r="C6381" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6382" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6382" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B6382" s="9" t="s">
+        <v>327</v>
+      </c>
+      <c r="C6382" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6383" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6383" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6383" s="9"/>
+      <c r="C6383" s="10"/>
+    </row>
+    <row r="6384" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6384" s="18">
+        <v>4.2</v>
+      </c>
+      <c r="B6384" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="C6384" s="10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6385" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6385" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B6385" s="9"/>
+      <c r="C6385" s="10" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="6386" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6386" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B6386" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6386" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6387" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6387" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6387" s="20"/>
+      <c r="C6387" s="22"/>
+    </row>
+    <row r="6432" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6432" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="B6432" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6432" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6433" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6433" s="4"/>
+      <c r="B6433" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6433" s="25"/>
+    </row>
+    <row r="6434" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6434" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6434" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6434" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6435" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6435" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6435" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6435" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6436" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6436" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6436" s="9"/>
+      <c r="C6436" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6437" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6437" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6437" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6437" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6438" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6438" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6438" s="9"/>
+      <c r="C6438" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6439" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6439" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6439" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6439" s="10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6440" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6440" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6440" s="9"/>
+      <c r="C6440" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6441" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B6441" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6441" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6442" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6442" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6442" s="9"/>
+      <c r="C6442" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6443" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6443" s="8"/>
+      <c r="B6443" s="9"/>
+      <c r="C6443" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="6444" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6444" s="8"/>
+      <c r="B6444" s="9"/>
+      <c r="C6444" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6445" s="8"/>
+      <c r="B6445" s="9"/>
+      <c r="C6445" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6446" s="8"/>
+      <c r="B6446" s="9"/>
+      <c r="C6446" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6447" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6447" s="8"/>
+      <c r="B6447" s="9"/>
+      <c r="C6447" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="6448" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6448" s="8"/>
+      <c r="B6448" s="9"/>
+      <c r="C6448" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6449" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6449" s="8"/>
+      <c r="B6449" s="9"/>
+      <c r="C6449" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="6450" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6450" s="8"/>
+      <c r="B6450" s="9"/>
+      <c r="C6450" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="6451" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6451" s="8"/>
+      <c r="B6451" s="9"/>
+      <c r="C6451" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6452" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6452" s="8"/>
+      <c r="B6452" s="9"/>
+      <c r="C6452" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="6453" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6453" s="8"/>
+      <c r="B6453" s="9"/>
+      <c r="C6453" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="6454" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6454" s="8"/>
+      <c r="B6454" s="9"/>
+      <c r="C6454" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6455" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6455" s="8"/>
+      <c r="B6455" s="9"/>
+      <c r="C6455" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="6456" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6456" s="8"/>
+      <c r="B6456" s="9"/>
+      <c r="C6456" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="6457" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6457" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6457" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6457" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6458" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6458" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6458" s="20"/>
+      <c r="C6458" s="22"/>
+    </row>
+    <row r="6491" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6491" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="B6491" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6491" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6492" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6492" s="4"/>
+      <c r="B6492" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6492" s="32"/>
+    </row>
+    <row r="6493" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6493" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6493" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6493" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6494" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6494" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6494" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6494" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6495" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6495" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6495" s="9"/>
+      <c r="C6495" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6496" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6496" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6496" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6496" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6497" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6497" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6497" s="9"/>
+      <c r="C6497" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6498" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6498" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6498" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6498" s="10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6499" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6499" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6499" s="9"/>
+      <c r="C6499" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6500" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6500" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B6500" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6500" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6501" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6501" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6501" s="9"/>
+      <c r="C6501" s="10"/>
+    </row>
+    <row r="6502" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6502" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6502" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6502" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6503" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6503" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B6503" s="9"/>
+      <c r="C6503" s="30" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6504" s="8"/>
+      <c r="B6504" s="9"/>
+      <c r="C6504" s="30"/>
+    </row>
+    <row r="6505" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6505" s="18">
+        <v>5.2</v>
+      </c>
+      <c r="B6505" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6505" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6506" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6506" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B6506" s="9"/>
+      <c r="C6506" s="10"/>
+    </row>
+    <row r="6507" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6507" s="8">
+        <v>6.2</v>
+      </c>
+      <c r="B6507" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6507" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6508" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6508" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6508" s="20"/>
+      <c r="C6508" s="22"/>
+    </row>
+    <row r="6550" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6550" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B6550" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6550" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6551" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6551" s="4"/>
+      <c r="B6551" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6551" s="25"/>
+    </row>
+    <row r="6552" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6552" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6552" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6552" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6553" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6553" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6553" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6553" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6554" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6554" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B6554" s="9"/>
+      <c r="C6554" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6555" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6555" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B6555" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6555" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6556" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6556" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B6556" s="9"/>
+      <c r="C6556" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6557" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B6557" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6557" s="10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="6558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6558" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B6558" s="9"/>
+      <c r="C6558" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6559" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B6559" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6559" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6560" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B6560" s="9"/>
+      <c r="C6560" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6561" s="18">
+        <v>4.2</v>
+      </c>
+      <c r="B6561" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6561" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6562" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B6562" s="9"/>
+      <c r="C6562" s="10" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="6563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6563" s="8"/>
+      <c r="B6563" s="9"/>
+      <c r="C6563" s="10" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="6564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6564" s="8"/>
+      <c r="B6564" s="9"/>
+      <c r="C6564" s="10" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6565" s="8"/>
+      <c r="B6565" s="9"/>
+      <c r="C6565" s="10" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6566" s="8"/>
+      <c r="B6566" s="9"/>
+      <c r="C6566" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="6567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6567" s="8"/>
+      <c r="B6567" s="9"/>
+      <c r="C6567" s="10" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="6568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6568" s="8"/>
+      <c r="B6568" s="9"/>
+      <c r="C6568" s="10" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6569" s="8"/>
+      <c r="B6569" s="9"/>
+      <c r="C6569" s="10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="6570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6570" s="8"/>
+      <c r="B6570" s="9"/>
+      <c r="C6570" s="10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="6571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6571" s="8"/>
+      <c r="B6571" s="9"/>
+      <c r="C6571" s="10" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6572" s="8"/>
+      <c r="B6572" s="9"/>
+      <c r="C6572" s="10" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="6573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6573" s="8"/>
+      <c r="B6573" s="9"/>
+      <c r="C6573" s="10" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="6574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6574" s="8"/>
+      <c r="B6574" s="9"/>
+      <c r="C6574" s="10" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6575" s="8"/>
+      <c r="B6575" s="9"/>
+      <c r="C6575" s="10" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="6576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6576" s="8"/>
+      <c r="B6576" s="9"/>
+      <c r="C6576" s="10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="6577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6577" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B6577" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6577" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6578" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6578" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6578" s="20"/>
+      <c r="C6578" s="22"/>
+    </row>
   </sheetData>
-  <mergeCells count="80">
+  <mergeCells count="85">
+    <mergeCell ref="C6031:C6032"/>
+    <mergeCell ref="C6147:C6148"/>
+    <mergeCell ref="B6492:C6492"/>
+    <mergeCell ref="C6503:C6504"/>
     <mergeCell ref="B5725:C5725"/>
+    <mergeCell ref="B6020:C6020"/>
     <mergeCell ref="B5607:C5607"/>
     <mergeCell ref="B5430:C5430"/>
     <mergeCell ref="B5489:C5489"/>

</xml_diff>

<commit_message>
Instructions up to 7B.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94886885-B220-4532-9DAD-FCA78D6CA6A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0228D394-E0DD-4A0C-8CED-D52FD7D6F380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -6854,6 +6854,12 @@
     <t>PLA (68)</t>
   </si>
   <si>
+    <t>ADC (69)</t>
+  </si>
+  <si>
+    <t>ROR (6A)</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Set </t>
     </r>
@@ -6866,6 +6872,27 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>A</t>
     </r>
     <r>
@@ -6876,6 +6903,375 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">.L &amp; $01). Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L = (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L &gt;&gt; 1) | (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &lt;&lt; 7). Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80) and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>RTL (6B)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Store as </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> by 3. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to (Operand + 1). Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to Bank.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read ((</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L | $0100)+3)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read u8(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L+2) | $0100</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Read u8(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>S</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L+1) | $0100</t>
+    </r>
+  </si>
+  <si>
+    <t>JMP (6C)</t>
+  </si>
+  <si>
+    <t>Absolute Indirect</t>
+  </si>
+  <si>
+    <t>Read Pointer</t>
+  </si>
+  <si>
+    <t>Read Pointer + 1</t>
+  </si>
+  <si>
+    <t>ADC (6D)</t>
+  </si>
+  <si>
+    <t>ROR (6E)</t>
+  </si>
+  <si>
+    <t>ADC (6F)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">.L to Operand.L. Set </t>
     </r>
     <r>
@@ -6960,509 +7356,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">.L. Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> to Operand. Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.H &amp; $80). Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>ADC (69)</t>
-  </si>
-  <si>
-    <t>ROR (6A)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.L &amp; $01). Perform </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L = (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L &gt;&gt; 1) | (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> &lt;&lt; 7). Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>N</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.L &amp; $80) and </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Z</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> based off </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>A</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>.L.</t>
     </r>
-  </si>
-  <si>
-    <t>RTL (6B)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Store as </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PB</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Inc. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> by 3. Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> to (Operand + 1). Set </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PB</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> to Bank.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Read ((</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L | $0100)+3)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Read u8(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L+2) | $0100</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Read u8(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>S</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.L+1) | $0100</t>
-    </r>
-  </si>
-  <si>
-    <t>JMP (6C)</t>
-  </si>
-  <si>
-    <t>Absolute Indirect</t>
-  </si>
-  <si>
-    <t>Read Pointer</t>
-  </si>
-  <si>
-    <t>Read Pointer + 1</t>
-  </si>
-  <si>
-    <t>ADC (6D)</t>
-  </si>
-  <si>
-    <t>ROR (6E)</t>
-  </si>
-  <si>
-    <t>ADC (6F)</t>
   </si>
 </sst>
 </file>
@@ -23938,36 +23833,31 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B6147" s="9"/>
-      <c r="C6147" s="35" t="s">
-        <v>315</v>
+      <c r="C6147" s="9" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="6148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6148" s="8"/>
-      <c r="B6148" s="9"/>
-      <c r="C6148" s="35"/>
+      <c r="A6148" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B6148" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6148" s="10" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="6149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6149" s="8">
-        <v>4.2</v>
-      </c>
-      <c r="B6149" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6149" s="10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6150" s="19" t="s">
+      <c r="A6149" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="B6150" s="20"/>
-      <c r="C6150" s="22"/>
+      <c r="B6149" s="20"/>
+      <c r="C6149" s="22"/>
     </row>
     <row r="6196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6196" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B6196" s="2" t="s">
         <v>22</v>
@@ -24152,7 +24042,7 @@
     </row>
     <row r="6255" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6255" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B6255" s="2" t="s">
         <v>22</v>
@@ -24216,7 +24106,7 @@
       </c>
       <c r="B6261" s="9"/>
       <c r="C6261" s="10" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6262" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -24239,7 +24129,7 @@
     </row>
     <row r="6314" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6314" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B6314" s="2" t="s">
         <v>6</v>
@@ -24319,7 +24209,7 @@
         <v>3.2</v>
       </c>
       <c r="B6323" s="9" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C6323" s="10" t="s">
         <v>180</v>
@@ -24337,7 +24227,7 @@
         <v>4.2</v>
       </c>
       <c r="B6325" s="9" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C6325" s="10" t="s">
         <v>45</v>
@@ -24355,10 +24245,10 @@
         <v>5.2</v>
       </c>
       <c r="B6327" s="9" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C6327" s="10" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6328" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -24367,7 +24257,7 @@
       </c>
       <c r="B6328" s="9"/>
       <c r="C6328" s="10" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6329" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -24390,7 +24280,7 @@
     </row>
     <row r="6373" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6373" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B6373" s="2" t="s">
         <v>19</v>
@@ -24402,7 +24292,7 @@
     <row r="6374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6374" s="4"/>
       <c r="B6374" s="24" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C6374" s="25"/>
     </row>
@@ -24482,7 +24372,7 @@
         <v>3.2</v>
       </c>
       <c r="B6382" s="9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C6382" s="10" t="s">
         <v>16</v>
@@ -24500,7 +24390,7 @@
         <v>4.2</v>
       </c>
       <c r="B6384" s="9" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C6384" s="10" t="s">
         <v>278</v>
@@ -24535,7 +24425,7 @@
     </row>
     <row r="6432" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6432" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B6432" s="2" t="s">
         <v>24</v>
@@ -24760,7 +24650,7 @@
     </row>
     <row r="6491" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6491" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B6491" s="2" t="s">
         <v>6</v>
@@ -24928,7 +24818,7 @@
     </row>
     <row r="6550" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6550" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B6550" s="2" t="s">
         <v>19</v>
@@ -25172,9 +25062,8 @@
       <c r="C6578" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="85">
+  <mergeCells count="84">
     <mergeCell ref="C6031:C6032"/>
-    <mergeCell ref="C6147:C6148"/>
     <mergeCell ref="B6492:C6492"/>
     <mergeCell ref="C6503:C6504"/>
     <mergeCell ref="B5725:C5725"/>

</xml_diff>

<commit_message>
Instructions up to 80.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0228D394-E0DD-4A0C-8CED-D52FD7D6F380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC99B2E1-C349-4ECD-AFA6-2A029381FD73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -7232,9 +7232,6 @@
     <t>JMP (6C)</t>
   </si>
   <si>
-    <t>Absolute Indirect</t>
-  </si>
-  <si>
     <t>Read Pointer</t>
   </si>
   <si>
@@ -7358,6 +7355,9 @@
       </rPr>
       <t>.L.</t>
     </r>
+  </si>
+  <si>
+    <t>Absolute Indirect (Jump)</t>
   </si>
 </sst>
 </file>
@@ -23834,7 +23834,7 @@
       </c>
       <c r="B6147" s="9"/>
       <c r="C6147" s="9" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="6148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -24292,7 +24292,7 @@
     <row r="6374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6374" s="4"/>
       <c r="B6374" s="24" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="C6374" s="25"/>
     </row>
@@ -24372,7 +24372,7 @@
         <v>3.2</v>
       </c>
       <c r="B6382" s="9" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C6382" s="10" t="s">
         <v>16</v>
@@ -24390,7 +24390,7 @@
         <v>4.2</v>
       </c>
       <c r="B6384" s="9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C6384" s="10" t="s">
         <v>278</v>
@@ -24425,7 +24425,7 @@
     </row>
     <row r="6432" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6432" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B6432" s="2" t="s">
         <v>24</v>
@@ -24650,7 +24650,7 @@
     </row>
     <row r="6491" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6491" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B6491" s="2" t="s">
         <v>6</v>
@@ -24818,7 +24818,7 @@
     </row>
     <row r="6550" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6550" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B6550" s="2" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Instructions up to 90.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCB5C5A1-2E7E-4F7C-803D-90B3BAB72959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE479A29-F3A7-4A31-9B1C-6F6FE0F62F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$7662</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$8496</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3270" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3557" uniqueCount="398">
   <si>
     <t>BRK (00)</t>
   </si>
@@ -7434,9 +7434,6 @@
     <t>ADC (77)</t>
   </si>
   <si>
-    <t>CLI (78)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Sets the </t>
     </r>
@@ -7932,6 +7929,675 @@
       </rPr>
       <t>.L.</t>
     </r>
+  </si>
+  <si>
+    <t>Program Counter Relative Long</t>
+  </si>
+  <si>
+    <t>SEI (78)</t>
+  </si>
+  <si>
+    <t>BRL (82)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> += Operand.</t>
+    </r>
+  </si>
+  <si>
+    <t>STA (83)</t>
+  </si>
+  <si>
+    <t>Stack Relative (Write)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Sets Operand to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>STY (84)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>STA (85)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>STX (86)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>STA (87)</t>
+  </si>
+  <si>
+    <t>Direct Indirect Long (Write)</t>
+  </si>
+  <si>
+    <t>DEY (88)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L -= 1, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>BIT (89)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L &amp; Operand.L).</t>
+    </r>
+  </si>
+  <si>
+    <t>TXA (8A)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Perform </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L = </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L, set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>N</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.L &amp; $80), set </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Z</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> based off </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.L.</t>
+    </r>
+  </si>
+  <si>
+    <t>PHB (8B)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Push </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> onto stack.</t>
+    </r>
+  </si>
+  <si>
+    <t>STY (8C)</t>
+  </si>
+  <si>
+    <t>Absolute (Write)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Sets Operand to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Y</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>STA (8D)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Sets Operand to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>STX (8E)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Inc </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Sets Operand to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>STA (8F)</t>
+  </si>
+  <si>
+    <t>Absolute Long (Write)</t>
+  </si>
+  <si>
+    <t>Write to Address:Bank</t>
   </si>
 </sst>
 </file>
@@ -8532,7 +9198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{236A51FB-68FA-4644-A8C6-D47AA32EBCC5}">
-  <dimension ref="A1:C7632"/>
+  <dimension ref="A1:C8452"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.7109375" customWidth="1"/>
@@ -23166,10 +23832,10 @@
     </row>
     <row r="5784" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5784" s="4"/>
-      <c r="B5784" s="24" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5784" s="25"/>
+      <c r="B5784" s="30" t="s">
+        <v>365</v>
+      </c>
+      <c r="C5784" s="31"/>
     </row>
     <row r="5785" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5785" s="12" t="s">
@@ -27480,7 +28146,7 @@
     </row>
     <row r="7081" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7081" s="1" t="s">
-        <v>342</v>
+        <v>366</v>
       </c>
       <c r="B7081" s="2" t="s">
         <v>22</v>
@@ -27544,7 +28210,7 @@
       </c>
       <c r="B7087" s="9"/>
       <c r="C7087" s="10" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7088" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -27567,7 +28233,7 @@
     </row>
     <row r="7140" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7140" s="1" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="B7140" s="2" t="s">
         <v>24</v>
@@ -27834,7 +28500,7 @@
     </row>
     <row r="7199" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7199" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B7199" s="2" t="s">
         <v>24</v>
@@ -27927,7 +28593,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B7209" s="33" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C7209" s="10"/>
     </row>
@@ -27961,7 +28627,7 @@
     </row>
     <row r="7258" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7258" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B7258" s="2" t="s">
         <v>22</v>
@@ -28025,7 +28691,7 @@
       </c>
       <c r="B7264" s="9"/>
       <c r="C7264" s="10" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7265" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -28048,7 +28714,7 @@
     </row>
     <row r="7317" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7317" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B7317" s="2" t="s">
         <v>6</v>
@@ -28060,7 +28726,7 @@
     <row r="7318" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7318" s="4"/>
       <c r="B7318" s="30" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C7318" s="31"/>
     </row>
@@ -28132,7 +28798,7 @@
       </c>
       <c r="B7325" s="9"/>
       <c r="C7325" s="10" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7326" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -28172,7 +28838,7 @@
         <v>5.2</v>
       </c>
       <c r="B7330" s="9" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C7330" s="10" t="s">
         <v>277</v>
@@ -28207,7 +28873,7 @@
     </row>
     <row r="7376" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7376" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="B7376" s="2" t="s">
         <v>24</v>
@@ -28291,7 +28957,7 @@
       </c>
       <c r="B7384" s="9"/>
       <c r="C7384" s="10" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7385" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -28474,7 +29140,7 @@
     </row>
     <row r="7435" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7435" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B7435" s="2" t="s">
         <v>98</v>
@@ -28670,7 +29336,7 @@
     </row>
     <row r="7494" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7494" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B7494" s="2" t="s">
         <v>19</v>
@@ -28929,7 +29595,7 @@
     </row>
     <row r="7553" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7553" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="B7553" s="2" t="s">
         <v>15</v>
@@ -28973,7 +29639,7 @@
       </c>
       <c r="B7557" s="9"/>
       <c r="C7557" s="10" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -29055,7 +29721,7 @@
     </row>
     <row r="7612" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7612" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B7612" s="2" t="s">
         <v>6</v>
@@ -29067,7 +29733,7 @@
     <row r="7613" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7613" s="4"/>
       <c r="B7613" s="30" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C7613" s="31"/>
     </row>
@@ -29119,21 +29785,21 @@
       </c>
       <c r="B7618" s="9"/>
       <c r="C7618" s="10" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="7619" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7619" s="8"/>
       <c r="B7619" s="9"/>
       <c r="C7619" s="10" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7620" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7620" s="8"/>
       <c r="B7620" s="9"/>
       <c r="C7620" s="10" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="7621" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -29203,7 +29869,7 @@
       </c>
       <c r="B7628" s="9"/>
       <c r="C7628" s="10" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="7629" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -29211,7 +29877,7 @@
         <v>6.2</v>
       </c>
       <c r="B7629" s="9" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C7629" s="10" t="s">
         <v>47</v>
@@ -29242,9 +29908,1677 @@
       <c r="B7632" s="20"/>
       <c r="C7632" s="22"/>
     </row>
+    <row r="7671" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7671" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B7671" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7671" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7672" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7672" s="4"/>
+      <c r="B7672" s="30" t="s">
+        <v>365</v>
+      </c>
+      <c r="C7672" s="31"/>
+    </row>
+    <row r="7673" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7673" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7673" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7673" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7674" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7674" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7674" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7674" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7675" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7675" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7675" s="9"/>
+      <c r="C7675" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7676" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7676" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B7676" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7676" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7677" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7677" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B7677" s="9"/>
+      <c r="C7677" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7678" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7678" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7678" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7678" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7679" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7679" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B7679" s="9"/>
+      <c r="C7679" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7680" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7680" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B7680" s="9"/>
+      <c r="C7680" s="10"/>
+    </row>
+    <row r="7681" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7681" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7681" s="9"/>
+      <c r="C7681" s="10" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="7682" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7682" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B7682" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7682" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7683" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7683" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7683" s="20"/>
+      <c r="C7683" s="22"/>
+    </row>
+    <row r="7730" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7730" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B7730" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7730" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7731" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7731" s="4"/>
+      <c r="B7731" s="24" t="s">
+        <v>370</v>
+      </c>
+      <c r="C7731" s="25"/>
+    </row>
+    <row r="7732" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7732" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7732" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7732" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7733" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7733" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7733" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7733" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7734" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7734" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7734" s="9"/>
+      <c r="C7734" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7735" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7735" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B7735" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7735" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7736" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7736" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B7736" s="9"/>
+      <c r="C7736" s="10" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="7737" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7737" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7737" s="9"/>
+      <c r="C7737" s="10"/>
+    </row>
+    <row r="7738" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7738" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B7738" s="9"/>
+      <c r="C7738" s="10" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="7739" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7739" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B7739" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7739" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7740" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7740" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7740" s="9"/>
+      <c r="C7740" s="10"/>
+    </row>
+    <row r="7741" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7741" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B7741" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7741" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7742" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7742" s="20"/>
+      <c r="C7742" s="22"/>
+    </row>
+    <row r="7789" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7789" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="B7789" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7789" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7790" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7790" s="4"/>
+      <c r="B7790" s="24" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7790" s="25"/>
+    </row>
+    <row r="7791" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7791" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7791" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7791" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7792" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7792" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7792" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7792" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7793" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7793" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7793" s="9"/>
+      <c r="C7793" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7794" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7794" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B7794" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7794" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7795" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7795" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B7795" s="16"/>
+      <c r="C7795" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7796" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7796" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7796" s="16"/>
+      <c r="C7796" s="23"/>
+    </row>
+    <row r="7797" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7797" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B7797" s="9"/>
+      <c r="C7797" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7798" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7798" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B7798" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7798" s="10" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="7799" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7799" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7799" s="9"/>
+      <c r="C7799" s="10"/>
+    </row>
+    <row r="7800" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7800" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B7800" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7800" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7801" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7801" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7801" s="20"/>
+      <c r="C7801" s="22"/>
+    </row>
+    <row r="7848" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7848" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B7848" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7848" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7849" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7849" s="4"/>
+      <c r="B7849" s="24" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7849" s="25"/>
+    </row>
+    <row r="7850" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7850" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7850" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7850" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7851" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7851" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7851" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7851" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7852" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7852" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7852" s="9"/>
+      <c r="C7852" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7853" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7853" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B7853" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7853" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7854" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B7854" s="16"/>
+      <c r="C7854" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7855" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7855" s="16"/>
+      <c r="C7855" s="23"/>
+    </row>
+    <row r="7856" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7856" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B7856" s="9"/>
+      <c r="C7856" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7857" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7857" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B7857" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7857" s="10" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="7858" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7858" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7858" s="9"/>
+      <c r="C7858" s="10"/>
+    </row>
+    <row r="7859" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7859" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B7859" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7859" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7860" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7860" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7860" s="20"/>
+      <c r="C7860" s="22"/>
+    </row>
+    <row r="7907" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7907" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B7907" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7907" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7908" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7908" s="4"/>
+      <c r="B7908" s="24" t="s">
+        <v>307</v>
+      </c>
+      <c r="C7908" s="25"/>
+    </row>
+    <row r="7909" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7909" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7909" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7909" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7910" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7910" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7910" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7910" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7911" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7911" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7911" s="9"/>
+      <c r="C7911" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7912" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7912" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B7912" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7912" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7913" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7913" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B7913" s="16"/>
+      <c r="C7913" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7914" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7914" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7914" s="16"/>
+      <c r="C7914" s="23"/>
+    </row>
+    <row r="7915" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7915" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B7915" s="9"/>
+      <c r="C7915" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7916" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7916" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B7916" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7916" s="10" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="7917" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7917" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7917" s="9"/>
+      <c r="C7917" s="10"/>
+    </row>
+    <row r="7918" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7918" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B7918" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7918" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7919" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7919" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7919" s="20"/>
+      <c r="C7919" s="22"/>
+    </row>
+    <row r="7966" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7966" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="B7966" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7966" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7967" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7967" s="4"/>
+      <c r="B7967" s="24" t="s">
+        <v>379</v>
+      </c>
+      <c r="C7967" s="25"/>
+    </row>
+    <row r="7968" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7968" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7968" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7968" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7969" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7969" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7969" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7969" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7970" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7970" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B7970" s="9"/>
+      <c r="C7970" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7971" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7971" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B7971" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7971" s="10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7972" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7972" s="15">
+        <v>2.1</v>
+      </c>
+      <c r="B7972" s="16"/>
+      <c r="C7972" s="23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7973" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7973" s="15">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B7973" s="16"/>
+      <c r="C7973" s="23"/>
+    </row>
+    <row r="7974" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7974" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B7974" s="9"/>
+      <c r="C7974" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7975" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7975" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B7975" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7975" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7976" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7976" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B7976" s="9"/>
+      <c r="C7976" s="10"/>
+    </row>
+    <row r="7977" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7977" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B7977" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7977" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7978" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7978" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B7978" s="9"/>
+      <c r="C7978" s="10"/>
+    </row>
+    <row r="7979" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7979" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B7979" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7979" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7980" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7980" s="8">
+        <v>6.1</v>
+      </c>
+      <c r="B7980" s="9"/>
+      <c r="C7980" s="10" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="7981" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7981" s="18">
+        <v>6.2</v>
+      </c>
+      <c r="B7981" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7981" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7982" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7982" s="8">
+        <v>7.1</v>
+      </c>
+      <c r="B7982" s="9"/>
+      <c r="C7982" s="10"/>
+    </row>
+    <row r="7983" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7983" s="8">
+        <v>7.2</v>
+      </c>
+      <c r="B7983" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7983" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7984" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7984" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7984" s="20"/>
+      <c r="C7984" s="22"/>
+    </row>
+    <row r="8025" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8025" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="B8025" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8025" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8026" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8026" s="4"/>
+      <c r="B8026" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8026" s="25"/>
+    </row>
+    <row r="8027" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8027" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8027" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8027" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8028" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8028" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8028" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8028" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8029" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8029" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8029" s="9"/>
+      <c r="C8029" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8030" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8030" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B8030" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8030" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8031" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8031" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8031" s="9"/>
+      <c r="C8031" s="10" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="8032" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8032" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8032" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8032" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8033" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8033" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8033" s="20"/>
+      <c r="C8033" s="22"/>
+    </row>
+    <row r="8084" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8084" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="B8084" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8084" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8085" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8085" s="4"/>
+      <c r="B8085" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8085" s="25"/>
+    </row>
+    <row r="8086" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8086" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8086" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8086" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8087" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8087" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8087" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8087" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8088" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8088" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8088" s="9"/>
+      <c r="C8088" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8089" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8089" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B8089" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8089" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8090" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8090" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8090" s="9"/>
+      <c r="C8090" s="10" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="8091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8091" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8091" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8091" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8092" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8092" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8092" s="20"/>
+      <c r="C8092" s="22"/>
+    </row>
+    <row r="8143" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8143" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="B8143" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8143" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8144" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8144" s="4"/>
+      <c r="B8144" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8144" s="25"/>
+    </row>
+    <row r="8145" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8145" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8145" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8145" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8146" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8146" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8146" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8147" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8147" s="9"/>
+      <c r="C8147" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8148" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="B8148" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8148" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8149" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8149" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8149" s="9"/>
+      <c r="C8149" s="10" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="8150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8150" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8150" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8150" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8151" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8151" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8151" s="20"/>
+      <c r="C8151" s="22"/>
+    </row>
+    <row r="8202" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8202" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B8202" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8202" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8203" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8203" s="4"/>
+      <c r="B8203" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8203" s="25"/>
+    </row>
+    <row r="8204" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8204" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8204" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8204" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8205" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8205" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8205" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8205" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8206" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8206" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8206" s="9"/>
+      <c r="C8206" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8207" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8207" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B8207" s="9"/>
+      <c r="C8207" s="10"/>
+    </row>
+    <row r="8208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8208" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8208" s="9"/>
+      <c r="C8208" s="10"/>
+    </row>
+    <row r="8209" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8209" s="18">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8209" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="C8209" s="10" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="8210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8210" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B8210" s="9"/>
+      <c r="C8210" s="10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8211" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B8211" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8211" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8212" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8212" s="20"/>
+      <c r="C8212" s="22"/>
+    </row>
+    <row r="8261" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8261" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B8261" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8261" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8262" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8262" s="4"/>
+      <c r="B8262" s="24" t="s">
+        <v>389</v>
+      </c>
+      <c r="C8262" s="25"/>
+    </row>
+    <row r="8263" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8263" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8263" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8263" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8264" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8264" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8264" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8264" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8265" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8265" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8265" s="9"/>
+      <c r="C8265" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8266" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8266" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B8266" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8266" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8267" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8267" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8267" s="9"/>
+      <c r="C8267" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8268" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8268" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8268" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8268" s="10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8269" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8269" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B8269" s="9"/>
+      <c r="C8269" s="10" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="8270" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8270" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B8270" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8270" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8271" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8271" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B8271" s="9"/>
+      <c r="C8271" s="10"/>
+    </row>
+    <row r="8272" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8272" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B8272" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8272" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8273" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8273" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8273" s="20"/>
+      <c r="C8273" s="22"/>
+    </row>
+    <row r="8320" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8320" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B8320" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8320" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8321" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8321" s="4"/>
+      <c r="B8321" s="24" t="s">
+        <v>389</v>
+      </c>
+      <c r="C8321" s="25"/>
+    </row>
+    <row r="8322" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8322" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8322" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8322" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8323" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8323" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8323" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8323" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8324" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8324" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8324" s="9"/>
+      <c r="C8324" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8325" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8325" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B8325" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8325" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8326" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8326" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8326" s="9"/>
+      <c r="C8326" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8327" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8327" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8327" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8327" s="10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8328" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8328" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B8328" s="9"/>
+      <c r="C8328" s="10" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="8329" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8329" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B8329" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8329" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8330" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8330" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B8330" s="9"/>
+      <c r="C8330" s="10"/>
+    </row>
+    <row r="8331" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8331" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B8331" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8331" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8332" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8332" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8332" s="20"/>
+      <c r="C8332" s="22"/>
+    </row>
+    <row r="8379" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8379" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B8379" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8379" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8380" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8380" s="4"/>
+      <c r="B8380" s="24" t="s">
+        <v>389</v>
+      </c>
+      <c r="C8380" s="25"/>
+    </row>
+    <row r="8381" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8381" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8381" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8381" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8382" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8382" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8382" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8382" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8383" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8383" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8383" s="9"/>
+      <c r="C8383" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8384" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8384" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B8384" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8384" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8385" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8385" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8385" s="9"/>
+      <c r="C8385" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8386" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8386" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8386" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8386" s="10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8387" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8387" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B8387" s="9"/>
+      <c r="C8387" s="10" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="8388" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8388" s="18">
+        <v>3.2</v>
+      </c>
+      <c r="B8388" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8388" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8389" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8389" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B8389" s="9"/>
+      <c r="C8389" s="10"/>
+    </row>
+    <row r="8390" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8390" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="B8390" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8390" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8391" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8391" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8391" s="20"/>
+      <c r="C8391" s="22"/>
+    </row>
+    <row r="8438" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8438" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="B8438" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8438" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8439" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8439" s="4"/>
+      <c r="B8439" s="24" t="s">
+        <v>396</v>
+      </c>
+      <c r="C8439" s="25"/>
+    </row>
+    <row r="8440" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8440" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8440" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8440" s="7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8441" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8441" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8441" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8441" s="11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8442" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8442" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="B8442" s="9"/>
+      <c r="C8442" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8443" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8443" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="B8443" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8443" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8444" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8444" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="B8444" s="9"/>
+      <c r="C8444" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8445" s="8">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="B8445" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8445" s="10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="8446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8446" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="B8446" s="9"/>
+      <c r="C8446" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8447" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8447" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="B8447" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8447" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8448" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8448" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="B8448" s="9"/>
+      <c r="C8448" s="10" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="8449" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8449" s="18">
+        <v>4.2</v>
+      </c>
+      <c r="B8449" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="C8449" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8450" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8450" s="8">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="B8450" s="9"/>
+      <c r="C8450" s="10"/>
+    </row>
+    <row r="8451" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8451" s="8">
+        <v>5.2</v>
+      </c>
+      <c r="B8451" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8451" s="10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8452" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8452" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8452" s="20"/>
+      <c r="C8452" s="22"/>
+    </row>
   </sheetData>
-  <mergeCells count="101">
+  <mergeCells count="103">
     <mergeCell ref="B7613:C7613"/>
+    <mergeCell ref="B5784:C5784"/>
+    <mergeCell ref="B7672:C7672"/>
     <mergeCell ref="C7451:C7452"/>
     <mergeCell ref="B7436:C7436"/>
     <mergeCell ref="C7558:C7559"/>

</xml_diff>